<commit_message>
Atualizacao automatica - 2026-08-26 12:00
</commit_message>
<xml_diff>
--- a/Ruas Triade.xlsx
+++ b/Ruas Triade.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Eder Azevedo\Desktop\Ata 2025 - 2027 Triade\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{462938BF-C7DE-4936-B5DB-D02E7241DF6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B691B473-AF61-4922-B91F-AB427DFB7D4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1560" yWindow="1560" windowWidth="15375" windowHeight="7785" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PLAN" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="41">
   <si>
     <t>Nome da Via</t>
   </si>
@@ -151,6 +151,9 @@
   </si>
   <si>
     <t>Rua Baia Grande</t>
+  </si>
+  <si>
+    <t>PARALISADA</t>
   </si>
 </sst>
 </file>
@@ -1114,7 +1117,7 @@
       </c>
       <c r="D11" s="13"/>
       <c r="E11" s="15" t="s">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="F11" s="16">
         <v>46259</v>

</xml_diff>

<commit_message>
Atualizacao automatica - 2026-08-26 12:01
</commit_message>
<xml_diff>
--- a/Ruas Triade.xlsx
+++ b/Ruas Triade.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Eder Azevedo\Desktop\Ata 2025 - 2027 Triade\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B691B473-AF61-4922-B91F-AB427DFB7D4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BA21D99-29AD-4DC3-A5BC-1B8536AF2CD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1560" yWindow="1560" windowWidth="15375" windowHeight="7785" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="40">
   <si>
     <t>Nome da Via</t>
   </si>
@@ -151,9 +151,6 @@
   </si>
   <si>
     <t>Rua Baia Grande</t>
-  </si>
-  <si>
-    <t>PARALISADA</t>
   </si>
 </sst>
 </file>
@@ -1117,7 +1114,7 @@
       </c>
       <c r="D11" s="13"/>
       <c r="E11" s="15" t="s">
-        <v>40</v>
+        <v>21</v>
       </c>
       <c r="F11" s="16">
         <v>46259</v>
@@ -1132,7 +1129,7 @@
         <v>3824629.24</v>
       </c>
       <c r="J11" s="19">
-        <v>0.05</v>
+        <v>0.25</v>
       </c>
       <c r="K11" s="20">
         <v>0</v>

</xml_diff>

<commit_message>
Atualizacao automatica - 2026-08-26 15:59
</commit_message>
<xml_diff>
--- a/Ruas Triade.xlsx
+++ b/Ruas Triade.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Eder Azevedo\Desktop\Ata 2025 - 2027 Triade\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BA21D99-29AD-4DC3-A5BC-1B8536AF2CD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB197E2F-DFE9-4454-A5F4-2A7C852DED75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1560" yWindow="1560" windowWidth="15375" windowHeight="7785" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1114,30 +1114,19 @@
       </c>
       <c r="D11" s="13"/>
       <c r="E11" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="F11" s="16">
-        <v>46259</v>
-      </c>
-      <c r="G11" s="16">
-        <v>46295</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="F11" s="16"/>
+      <c r="G11" s="16"/>
       <c r="H11" s="17">
         <v>12446</v>
       </c>
       <c r="I11" s="18">
         <v>3824629.24</v>
       </c>
-      <c r="J11" s="19">
-        <v>0.25</v>
-      </c>
-      <c r="K11" s="20">
-        <v>0</v>
-      </c>
-      <c r="L11" s="21">
-        <f>I11-K11</f>
-        <v>3824629.24</v>
-      </c>
+      <c r="J11" s="19"/>
+      <c r="K11" s="20"/>
+      <c r="L11" s="21"/>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" s="13"/>

</xml_diff>

<commit_message>
Atualizacao automatica - 2026-08-28 15:33
</commit_message>
<xml_diff>
--- a/Ruas Triade.xlsx
+++ b/Ruas Triade.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Eder Azevedo\Desktop\Ata 2025 - 2027 Triade\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB197E2F-DFE9-4454-A5F4-2A7C852DED75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A1BCF48-FB12-486F-B986-524F68749DBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="1560" windowWidth="15375" windowHeight="7785" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PLAN" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="46">
   <si>
     <t>Nome da Via</t>
   </si>
@@ -151,6 +151,24 @@
   </si>
   <si>
     <t>Rua Baia Grande</t>
+  </si>
+  <si>
+    <t>CEP/Endereco Inicial</t>
+  </si>
+  <si>
+    <t>CEP/Endereco Final</t>
+  </si>
+  <si>
+    <t>CEP/Endereco Inicial e Final = OPCIONAL. So preencher se a rua for nova e ainda nao existir mapeada (ex: loteamento novo).</t>
+  </si>
+  <si>
+    <t>Se a rua ja existir de verdade (mesmo sem obra iniciada), so o nome correto na coluna C ja e suficiente - o resto e feito automaticamente.</t>
+  </si>
+  <si>
+    <t>Formato aceito: CEP (ex: 03927-350) ou endereco (ex: Rua Estrela Guia, 100).</t>
+  </si>
+  <si>
+    <t>Rua Coelho Neto</t>
   </si>
 </sst>
 </file>
@@ -161,7 +179,7 @@
     <numFmt numFmtId="44" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="&quot;R$ &quot;#,##0.00"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -193,6 +211,13 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="9"/>
+      <color rgb="FF808080"/>
+      <name val="Calibri"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -251,7 +276,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -317,6 +342,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Moeda 2" xfId="2" xr:uid="{F764D4D9-EC85-4D1F-BB6B-E9AAAE726BF8}"/>
@@ -705,7 +731,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:N30"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
@@ -720,9 +746,10 @@
     <col min="10" max="10" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="19.28515625" style="11" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="14" width="26.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
@@ -759,8 +786,14 @@
       <c r="L1" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>11</v>
       </c>
@@ -798,7 +831,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>11</v>
       </c>
@@ -836,7 +869,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
@@ -874,7 +907,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>11</v>
       </c>
@@ -912,7 +945,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>11</v>
       </c>
@@ -950,7 +983,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>11</v>
       </c>
@@ -988,7 +1021,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>11</v>
       </c>
@@ -1026,7 +1059,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>11</v>
       </c>
@@ -1064,7 +1097,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>17</v>
       </c>
@@ -1104,7 +1137,7 @@
         <v>395633.60000000009</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="13"/>
       <c r="B11" s="14" t="s">
         <v>12</v>
@@ -1128,7 +1161,7 @@
       <c r="K11" s="20"/>
       <c r="L11" s="21"/>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="13"/>
       <c r="B12" s="14" t="s">
         <v>12</v>
@@ -1152,7 +1185,7 @@
       <c r="K12" s="20"/>
       <c r="L12" s="21"/>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="13"/>
       <c r="B13" s="14" t="s">
         <v>18</v>
@@ -1176,7 +1209,7 @@
       <c r="K13" s="20"/>
       <c r="L13" s="21"/>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="13"/>
       <c r="B14" s="14" t="s">
         <v>18</v>
@@ -1200,7 +1233,7 @@
       <c r="K14" s="20"/>
       <c r="L14" s="21"/>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="13"/>
       <c r="B15" s="14" t="s">
         <v>18</v>
@@ -1224,7 +1257,7 @@
       <c r="K15" s="20"/>
       <c r="L15" s="21"/>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="13"/>
       <c r="B16" s="14" t="s">
         <v>18</v>
@@ -1298,14 +1331,24 @@
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" s="13"/>
-      <c r="B19" s="14"/>
-      <c r="C19" s="22"/>
+      <c r="B19" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="C19" s="22" t="s">
+        <v>45</v>
+      </c>
       <c r="D19" s="13"/>
-      <c r="E19" s="15"/>
+      <c r="E19" s="15" t="s">
+        <v>31</v>
+      </c>
       <c r="F19" s="16"/>
       <c r="G19" s="16"/>
-      <c r="H19" s="17"/>
-      <c r="I19" s="18"/>
+      <c r="H19" s="17">
+        <v>5000</v>
+      </c>
+      <c r="I19" s="18">
+        <v>1500000</v>
+      </c>
       <c r="J19" s="19"/>
       <c r="K19" s="20"/>
       <c r="L19" s="21"/>
@@ -1339,6 +1382,21 @@
         <v>29</v>
       </c>
     </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B28" s="25" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B29" s="25" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B30" s="25" t="s">
+        <v>44</v>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" sqref="E2:E20" xr:uid="{00000000-0002-0000-0000-000000000000}">

</xml_diff>

<commit_message>
Atualizacao planilha - Ruas Triade
</commit_message>
<xml_diff>
--- a/Ruas Triade.xlsx
+++ b/Ruas Triade.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Eder Azevedo\Desktop\Ata 2025 - 2027 Triade\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Eder Azevedo\Desktop\01.02.00020 - Ata PMSP 2025\03 - Projetos\00 Mapa Ruas Ata 020\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A1BCF48-FB12-486F-B986-524F68749DBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBB0B395-1FC8-41D5-87B2-C325BEC6689A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="44">
   <si>
     <t>Nome da Via</t>
   </si>
@@ -96,9 +96,6 @@
     <t>CONCLUIDA</t>
   </si>
   <si>
-    <t>EM EXECUÇÃO</t>
-  </si>
-  <si>
     <t>Travessa Paracelsus</t>
   </si>
   <si>
@@ -166,9 +163,6 @@
   </si>
   <si>
     <t>Formato aceito: CEP (ex: 03927-350) ou endereco (ex: Rua Estrela Guia, 100).</t>
-  </si>
-  <si>
-    <t>Rua Coelho Neto</t>
   </si>
 </sst>
 </file>
@@ -751,7 +745,7 @@
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>10</v>
@@ -787,10 +781,10 @@
         <v>9</v>
       </c>
       <c r="M1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="N1" s="1" t="s">
         <v>40</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
@@ -839,7 +833,7 @@
         <v>12</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D3" s="2">
         <v>120</v>
@@ -877,7 +871,7 @@
         <v>12</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D4" s="2">
         <v>120</v>
@@ -953,7 +947,7 @@
         <v>12</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D6" s="2">
         <v>120</v>
@@ -991,7 +985,7 @@
         <v>12</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D7" s="2">
         <v>120</v>
@@ -1111,7 +1105,7 @@
         <v>90</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F10" s="4">
         <v>46206</v>
@@ -1126,15 +1120,14 @@
         <v>1987651.67</v>
       </c>
       <c r="J10" s="6">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="K10" s="12">
-        <f>1987651.67-395633.6</f>
-        <v>1592018.0699999998</v>
+        <f>I10-200000</f>
+        <v>1787651.67</v>
       </c>
       <c r="L10" s="7">
-        <f>I10-K10</f>
-        <v>395633.60000000009</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
@@ -1143,11 +1136,11 @@
         <v>12</v>
       </c>
       <c r="C11" s="22" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D11" s="13"/>
       <c r="E11" s="15" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F11" s="16"/>
       <c r="G11" s="16"/>
@@ -1167,11 +1160,11 @@
         <v>12</v>
       </c>
       <c r="C12" s="22" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D12" s="13"/>
       <c r="E12" s="15" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F12" s="16"/>
       <c r="G12" s="16"/>
@@ -1191,11 +1184,11 @@
         <v>18</v>
       </c>
       <c r="C13" s="23" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D13" s="13"/>
       <c r="E13" s="15" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F13" s="16"/>
       <c r="G13" s="16"/>
@@ -1215,11 +1208,11 @@
         <v>18</v>
       </c>
       <c r="C14" s="23" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D14" s="13"/>
       <c r="E14" s="15" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F14" s="16"/>
       <c r="G14" s="16"/>
@@ -1239,11 +1232,11 @@
         <v>18</v>
       </c>
       <c r="C15" s="24" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D15" s="13"/>
       <c r="E15" s="15" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F15" s="16"/>
       <c r="G15" s="16"/>
@@ -1263,11 +1256,11 @@
         <v>18</v>
       </c>
       <c r="C16" s="22" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D16" s="13"/>
       <c r="E16" s="15" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F16" s="16"/>
       <c r="G16" s="16"/>
@@ -1284,14 +1277,14 @@
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" s="13"/>
       <c r="B17" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="C17" s="22" t="s">
         <v>36</v>
-      </c>
-      <c r="C17" s="22" t="s">
-        <v>37</v>
       </c>
       <c r="D17" s="13"/>
       <c r="E17" s="15" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F17" s="16"/>
       <c r="G17" s="16"/>
@@ -1308,14 +1301,14 @@
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" s="13"/>
       <c r="B18" s="14" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C18" s="22" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D18" s="13"/>
       <c r="E18" s="15" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F18" s="16"/>
       <c r="G18" s="16"/>
@@ -1331,24 +1324,14 @@
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" s="13"/>
-      <c r="B19" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="C19" s="22" t="s">
-        <v>45</v>
-      </c>
+      <c r="B19" s="14"/>
+      <c r="C19" s="22"/>
       <c r="D19" s="13"/>
-      <c r="E19" s="15" t="s">
-        <v>31</v>
-      </c>
+      <c r="E19" s="15"/>
       <c r="F19" s="16"/>
       <c r="G19" s="16"/>
-      <c r="H19" s="17">
-        <v>5000</v>
-      </c>
-      <c r="I19" s="18">
-        <v>1500000</v>
-      </c>
+      <c r="H19" s="17"/>
+      <c r="I19" s="18"/>
       <c r="J19" s="19"/>
       <c r="K19" s="20"/>
       <c r="L19" s="21"/>
@@ -1369,32 +1352,32 @@
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B24" s="8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B25" s="8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B28" s="25" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B29" s="25" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B30" s="25" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>